<commit_message>
feat: Update SQL batch file for day 10 and add new file for day 11.
</commit_message>
<xml_diff>
--- a/batches/24/day_10.xlsx
+++ b/batches/24/day_10.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ac217573afc2a6e8/Documents/work/acciojob/modules/sql/batches/24/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/batches/24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{14109102-90B0-AE48-8325-393F5E70DEE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D537760C-1F2D-AF42-AF41-2E523261E5A7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{967901B9-2288-D949-B9EF-9519566B6EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="2" xr2:uid="{7408A07C-E1A0-9243-8A39-627DBE53FE8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Recap" sheetId="1" r:id="rId1"/>
     <sheet name="Agenda" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Muti Join" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -38,6 +38,47 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Left join</t>
+  </si>
+  <si>
+    <t>customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">inner join </t>
+  </si>
+  <si>
+    <t>products</t>
+  </si>
+  <si>
+    <t>inner join</t>
+  </si>
+  <si>
+    <t>There will be some orders which have illegal cust_id</t>
+  </si>
+  <si>
+    <t>There will be customers who never placed any order</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>inner</t>
+  </si>
+  <si>
+    <t>Orders with legal cust_id</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -177,6 +218,99 @@
         <a:xfrm>
           <a:off x="825500" y="203200"/>
           <a:ext cx="7772400" cy="5336759"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>812800</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{69EC8A97-C271-5EB9-4D32-9E8D92722B31}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7404100" cy="647700"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>355600</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>148872</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2AA6FEA6-C56B-8076-38EA-17E46BE451A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="2438400"/>
+          <a:ext cx="7772400" cy="5025672"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -527,10 +661,61 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501DD535-2F4C-9446-BEC2-A13FA3E6DA26}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6AE770BB-F036-6443-80C6-F8C435CA762E}">
+  <dimension ref="A6:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="43.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>